<commit_message>
Fix Excel collapsible outline controls after column deletions
Stale outline metadata on deleted DCF columns L/M and Revenue Drivers
column L broke +/- click targets in Excel. Updated restore_outline_groups
to clear outlines before reapplying, keep Source column C visible, group
only empty B/D doc columns, fix NOPAT summary row 41 visibility, and put
the DCF WC +/- control on row 19 (summaryBelow=False).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -1115,14 +1115,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="B2:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1130,7 +1129,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1145,7 +1143,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1153,7 +1150,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1175,7 +1171,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -1197,7 +1192,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="5" t="inlineStr">
         <is>
@@ -1205,7 +1199,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="11" t="inlineStr">
         <is>
@@ -1233,7 +1226,7 @@
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
-    <col hidden="1" outlineLevel="1" width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col hidden="1" outlineLevel="1" width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1314,7 +1307,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1422,7 +1414,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1632,7 +1623,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1668,7 +1658,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -1756,7 +1745,7 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
-    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col hidden="1" outlineLevel="1" width="38" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -2232,7 +2221,6 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4235,7 +4223,6 @@
         <v/>
       </c>
     </row>
-    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4293,7 +4280,6 @@
         <v/>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4301,7 +4287,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -5383,10 +5368,10 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col hidden="1" outlineLevel="1" width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
     <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="10" max="10"/>
     <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="11" max="11"/>
-    <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5551,7 +5536,11 @@
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="K7" s="19" t="n"/>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="41" t="inlineStr">
@@ -5585,7 +5574,11 @@
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="K8" s="19" t="n"/>
+      <c r="K8" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
@@ -5701,7 +5694,11 @@
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="K11" s="19" t="n"/>
+      <c r="K11" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
@@ -5735,7 +5732,11 @@
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="K12" s="19" t="n"/>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="61" t="inlineStr">
@@ -5851,7 +5852,11 @@
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="K15" s="19" t="n"/>
+      <c r="K15" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
@@ -5885,7 +5890,11 @@
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="K16" s="19" t="n"/>
+      <c r="K16" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="61" t="inlineStr">
@@ -5999,7 +6008,11 @@
           <t>FY2025 10-K: sales per square foot</t>
         </is>
       </c>
-      <c r="K19" s="19" t="n"/>
+      <c r="K19" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="41" t="inlineStr">
@@ -6043,7 +6056,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6135,7 +6147,11 @@
           <t>FY2025 10-K: comparable sales &amp; SPSF</t>
         </is>
       </c>
-      <c r="K24" s="19" t="n"/>
+      <c r="K24" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
@@ -6172,7 +6188,11 @@
           <t>FY2025 10-K: Americas comparable sales</t>
         </is>
       </c>
-      <c r="K25" s="19" t="n"/>
+      <c r="K25" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="41" t="inlineStr">
@@ -6209,7 +6229,11 @@
           <t>FY2025 10-K: China Mainland comparable sales</t>
         </is>
       </c>
-      <c r="K26" s="19" t="n"/>
+      <c r="K26" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="41" t="inlineStr">
@@ -6246,7 +6270,11 @@
           <t>FY2025 10-K: Rest of World comparable sales</t>
         </is>
       </c>
-      <c r="K27" s="19" t="n"/>
+      <c r="K27" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="41" t="inlineStr">
@@ -6428,7 +6456,11 @@
           <t>FY2025 10-K: store traffic commentary</t>
         </is>
       </c>
-      <c r="K32" s="19" t="n"/>
+      <c r="K32" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="41" t="n"/>
@@ -6456,7 +6488,11 @@
           <t>FY2025 10-K: conversion rate commentary</t>
         </is>
       </c>
-      <c r="K33" s="19" t="n"/>
+      <c r="K33" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="41" t="n"/>
@@ -6484,9 +6520,12 @@
           <t>FY2025 10-K: average order value commentary</t>
         </is>
       </c>
-      <c r="K34" s="19" t="n"/>
-    </row>
-    <row r="35"/>
+      <c r="K34" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -6578,7 +6617,11 @@
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="K38" s="19" t="n"/>
+      <c r="K38" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="41" t="inlineStr">
@@ -6610,7 +6653,11 @@
           <t>FY2025 10-K: digital / traffic commentary</t>
         </is>
       </c>
-      <c r="K39" s="19" t="n"/>
+      <c r="K39" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="41" t="inlineStr">
@@ -6642,7 +6689,11 @@
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="K40" s="19" t="n"/>
+      <c r="K40" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="61" t="inlineStr">
@@ -6680,7 +6731,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -6777,7 +6827,11 @@
           <t>FY2025 10-K: channel revenue table</t>
         </is>
       </c>
-      <c r="K45" s="19" t="n"/>
+      <c r="K45" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="70" customHeight="1">
       <c r="A46" s="41" t="inlineStr">
@@ -6819,7 +6873,11 @@
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="K46" s="19" t="n"/>
+      <c r="K46" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="70" customHeight="1">
       <c r="A47" s="41" t="inlineStr">
@@ -6861,7 +6919,11 @@
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="K47" s="19" t="n"/>
+      <c r="K47" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="70" customHeight="1">
       <c r="A48" s="41" t="inlineStr">
@@ -6903,7 +6965,11 @@
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="K48" s="19" t="n"/>
+      <c r="K48" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="28" customHeight="1">
       <c r="A49" s="41" t="inlineStr">
@@ -6935,7 +7001,11 @@
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="K49" s="19" t="n"/>
+      <c r="K49" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="41" t="inlineStr">
@@ -6967,7 +7037,11 @@
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="K50" s="19" t="n"/>
+      <c r="K50" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="41" t="inlineStr">
@@ -6999,9 +7073,12 @@
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="K51" s="19" t="n"/>
-    </row>
-    <row r="52"/>
+      <c r="K51" s="19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
+    </row>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -7127,6 +7204,11 @@
       <c r="J56" s="18" t="inlineStr">
         <is>
           <t>Scenarios tab: base revenue</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>'Scenarios'!G25</t>
         </is>
       </c>
     </row>
@@ -7264,7 +7346,7 @@
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col hidden="1" outlineLevel="1" width="22" customWidth="1" min="2" max="2"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -7339,7 +7421,6 @@
     <row r="4">
       <c r="A4" s="26" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -7542,7 +7623,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -8336,7 +8416,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+    <row r="41" ht="28" customHeight="1">
       <c r="A41" s="23" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT</t>
@@ -8370,7 +8450,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="61" t="inlineStr">
         <is>
@@ -8446,7 +8525,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J104"/>
@@ -8454,7 +8533,7 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
-    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -8463,8 +8542,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
-    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="12" max="12"/>
-    <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -8536,7 +8615,11 @@
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="38" t="n"/>
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>LULU_Assumptions_Memo.pdf</t>
+        </is>
+      </c>
       <c r="C4" s="85" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab</t>
@@ -9604,7 +9687,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="n"/>
     </row>
@@ -9819,8 +9901,6 @@
         <v/>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -9839,7 +9919,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -9900,7 +9979,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -9985,7 +10063,6 @@
         <v/>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -10106,7 +10183,6 @@
         <v/>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -10167,7 +10243,6 @@
         <v/>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -10246,7 +10321,6 @@
         <v/>
       </c>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -10353,8 +10427,6 @@
       </c>
       <c r="D94" s="26" t="n"/>
     </row>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -10614,7 +10686,7 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
-    <col hidden="1" outlineLevel="1" width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col hidden="1" outlineLevel="1" width="44" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -10775,7 +10847,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -11093,7 +11164,6 @@
         <v>407521</v>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="n"/>
     </row>
@@ -11171,7 +11241,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -11222,7 +11291,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -11312,7 +11380,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -11459,7 +11526,6 @@
         <v/>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix formula error popups and frozen Excel outline controls
- Convert NOPAT Bridge subtotal labels from invalid formulas to plain text
- Restore DCF/Revenue Drivers internal hyperlinks (were sheet-ref strings)
- Remove broken non-contiguous B/D column groups; keep row groups and RD J-K
- Clear stale outline metadata on all sheets before reapplying groups

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -1225,9 +1225,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1744,9 +1744,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -7208,7 +7208,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>'Scenarios'!G25</t>
+          <t>Scenarios tab: base revenue</t>
         </is>
       </c>
     </row>
@@ -7345,9 +7345,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col hidden="1" outlineLevel="1" width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -7421,6 +7421,7 @@
     <row r="4">
       <c r="A4" s="26" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -7623,6 +7624,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -7802,9 +7804,10 @@
       </c>
     </row>
     <row r="21" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A21" s="23">
-        <f> Adjusted EBIT (Phase 1)</f>
-        <v/>
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>Adjusted EBIT (Phase 1)</t>
+        </is>
       </c>
       <c r="B21" s="17" t="n"/>
       <c r="C21" s="24" t="inlineStr">
@@ -7943,9 +7946,10 @@
       </c>
     </row>
     <row r="26" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A26" s="23">
-        <f> EBIT after lease &amp; capitalization (Phase 2)</f>
-        <v/>
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>EBIT after lease &amp; capitalization (Phase 2)</t>
+        </is>
       </c>
       <c r="B26" s="17" t="n"/>
       <c r="C26" s="24" t="inlineStr">
@@ -8239,9 +8243,10 @@
       </c>
     </row>
     <row r="35" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A35" s="23">
-        <f> EBIT after channel mix (Phase 3)</f>
-        <v/>
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>EBIT after channel mix (Phase 3)</t>
+        </is>
       </c>
       <c r="B35" s="17" t="n"/>
       <c r="C35" s="24" t="inlineStr">
@@ -8275,9 +8280,10 @@
       </c>
     </row>
     <row r="36" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A36" s="23">
-        <f> Normalized EBIT (tax base for NOPAT)</f>
-        <v/>
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>Normalized EBIT (tax base for NOPAT)</t>
+        </is>
       </c>
       <c r="B36" s="17" t="n"/>
       <c r="C36" s="24" t="inlineStr">
@@ -8450,6 +8456,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="61" t="inlineStr">
         <is>
@@ -8532,9 +8539,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -8627,7 +8634,7 @@
       </c>
       <c r="D4" s="85" t="inlineStr">
         <is>
-          <t>'Revenue Drivers'!A1</t>
+          <t>Revenue Drivers tab</t>
         </is>
       </c>
     </row>
@@ -10685,9 +10692,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>

</xml_diff>

<commit_message>
Fix outline groups not expanding: set collapsed on summary rows/cols
Excel requires collapsed=True on the summary row/column (DCF row 19,
NOPAT row 41, Revenue Drivers col L) for +/- controls to toggle hidden
detail rows/cols. Also use column_dimensions.group() for contiguous J-K.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -5369,9 +5369,8 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="10" max="10"/>
-    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="10" max="11"/>
+    <col collapsed="1" width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8422,7 +8421,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
+    <row r="41" collapsed="1" ht="28" customHeight="1">
       <c r="A41" s="23" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT</t>
@@ -9072,7 +9071,7 @@
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" collapsed="1">
       <c r="A19" s="52" t="inlineStr">
         <is>
           <t>Working capital schedule (driver-based) [click − to collapse detail]</t>

</xml_diff>

<commit_message>
Remove GIS IR selection assignment line from Cover page
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -1115,13 +1115,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1129,6 +1130,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1143,6 +1145,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1150,6 +1153,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1171,6 +1175,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -1192,6 +1197,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="5" t="inlineStr">
         <is>
@@ -1199,12 +1205,9 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Built from scratch for the GIS IR selection assignment.</t>
-        </is>
-      </c>
+      <c r="B19" s="11" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1"/>
     <row r="21" ht="36" customHeight="1"/>
@@ -7420,7 +7423,6 @@
     <row r="4">
       <c r="A4" s="26" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -7623,7 +7625,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -8455,7 +8456,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="61" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove LULU Assumptions PDF references from Cover and DCF tabs
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -1191,11 +1191,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>ASSUMPTIONS GUIDE (PDF — every tab)</t>
-        </is>
-      </c>
+      <c r="B15" s="5" t="n"/>
     </row>
     <row r="16"/>
     <row r="17" ht="36" customHeight="1">
@@ -1310,6 +1306,7 @@
         <v>0.3</v>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1417,6 +1414,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1626,6 +1624,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1661,6 +1660,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2224,6 +2224,7 @@
         <v>0.75</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4226,6 +4227,7 @@
         <v/>
       </c>
     </row>
+    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4283,6 +4285,7 @@
         <v/>
       </c>
     </row>
+    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4290,6 +4293,7 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -6058,6 +6062,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6528,6 +6533,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -6733,6 +6739,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -7081,6 +7088,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -7423,6 +7431,7 @@
     <row r="4">
       <c r="A4" s="26" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -7625,6 +7634,7 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -8456,6 +8466,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="61" t="inlineStr">
         <is>
@@ -8621,11 +8632,7 @@
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
-        <is>
-          <t>LULU_Assumptions_Memo.pdf</t>
-        </is>
-      </c>
+      <c r="A4" s="38" t="n"/>
       <c r="C4" s="85" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab</t>
@@ -9693,6 +9700,7 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="n"/>
     </row>
@@ -9907,6 +9915,8 @@
         <v/>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -9925,6 +9935,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -9985,6 +9996,7 @@
         <v/>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -10069,6 +10081,7 @@
         <v/>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -10189,6 +10202,7 @@
         <v/>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -10249,6 +10263,7 @@
         <v/>
       </c>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -10327,6 +10342,7 @@
         <v/>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -10433,6 +10449,8 @@
       </c>
       <c r="D94" s="26" t="n"/>
     </row>
+    <row r="95"/>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -10623,58 +10641,57 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
     <hyperlink ref="C4" location="'NOPAT Bridge'!A1"/>
     <hyperlink ref="D4" location="'Revenue Drivers'!A1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId33"/>
     <hyperlink ref="C30" location="'Scenarios'!A105"/>
     <hyperlink ref="C31" location="'Scenarios'!A110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId35"/>
     <hyperlink ref="C33" location="'Scenarios'!A120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId44"/>
     <hyperlink ref="C82" location="'DCF'!E46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId46"/>
     <hyperlink ref="C104" location="'Scenarios'!G9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10853,6 +10870,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -11170,6 +11188,7 @@
         <v>407521</v>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="n"/>
     </row>
@@ -11247,6 +11266,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -11297,6 +11317,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -11386,6 +11407,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -11532,6 +11554,7 @@
         <v/>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove assumptions memo row and update NOPAT Bridge tariff note
- Clear DCF row 4 (assumptions memo) and reset row height
- Replace NOPAT Bridge A44/A45 with single FY26 tariff/tax-path note

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="53">
+  <fonts count="54">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -346,6 +346,11 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -405,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -749,6 +754,9 @@
     </xf>
     <xf numFmtId="165" fontId="52" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1115,14 +1123,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="B2:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1130,7 +1137,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1145,7 +1151,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1153,7 +1158,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1175,7 +1179,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -1193,7 +1196,6 @@
     <row r="15">
       <c r="B15" s="5" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="5" t="inlineStr">
         <is>
@@ -1201,7 +1203,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="11" t="n"/>
     </row>
@@ -1306,7 +1307,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1414,7 +1414,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1624,7 +1623,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1660,7 +1658,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2224,7 +2221,6 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4227,7 +4223,6 @@
         <v/>
       </c>
     </row>
-    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4285,7 +4280,6 @@
         <v/>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4293,7 +4287,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -6062,7 +6055,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6533,7 +6525,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -6739,7 +6730,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -7088,7 +7078,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -7431,7 +7420,6 @@
     <row r="4">
       <c r="A4" s="26" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -7634,7 +7622,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -8466,7 +8453,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="61" t="inlineStr">
         <is>
@@ -8487,18 +8473,14 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="26" t="inlineStr">
-        <is>
-          <t>Steps 1–4: DCF unchanged on FY26. Step 5 changes NOPAT only (tax). Step 6 changes FY26 EBIT (+ tariff).</t>
+      <c r="A44" s="126" t="inlineStr">
+        <is>
+          <t>FY26 EBIT adjusted for one-time tariff refund. Base/Bear/Bull paths link to normalized NOPAT using a flat operating tax rate.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="26" t="inlineStr">
-        <is>
-          <t>Scenarios base-case NOPAT (col G) links to NORMALIZED NOPAT above. Bear/bull apply the same t_operating to their EBIT paths.</t>
-        </is>
-      </c>
+      <c r="A45" s="26" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -8631,7 +8613,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="38" t="n"/>
       <c r="C4" s="85" t="inlineStr">
         <is>
@@ -9700,7 +9682,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="n"/>
     </row>
@@ -9915,8 +9896,6 @@
         <v/>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -9935,7 +9914,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -9996,7 +9974,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -10081,7 +10058,6 @@
         <v/>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -10202,7 +10178,6 @@
         <v/>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -10263,7 +10238,6 @@
         <v/>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -10342,7 +10316,6 @@
         <v/>
       </c>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -10449,8 +10422,6 @@
       </c>
       <c r="D94" s="26" t="n"/>
     </row>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -10870,7 +10841,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -11188,7 +11158,6 @@
         <v>407521</v>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="n"/>
     </row>
@@ -11266,7 +11235,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -11317,7 +11285,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -11407,7 +11374,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -11554,7 +11520,6 @@
         <v/>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove NOPAT Bridge tab; wire DCF NOPAT directly from Scenarios
The bridge was a reconciliation memo only. Forecast NOPAT is now
EBIT × (1 − cash tax rate) on Scenarios; DCF tax and net income rows
link directly without the extra tab.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -11,9 +11,8 @@
     <sheet name="WACC" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DCF" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Comps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DCF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Comps" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1189,7 +1188,7 @@
     <row r="14">
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>WACC • Revenue Drivers • NOPAT Bridge • Scenarios • DCF • Comps / Football Field</t>
+          <t>WACC • Revenue Drivers • Scenarios • DCF • Comps / Football Field</t>
         </is>
       </c>
     </row>
@@ -2710,15 +2709,15 @@
         </is>
       </c>
       <c r="F50" s="42">
-        <f>F45*(1-'NOPAT Bridge'!F$39)</f>
+        <f>F45*(1-$G$11)</f>
         <v/>
       </c>
       <c r="G50" s="42">
-        <f>'NOPAT Bridge'!F41</f>
+        <f>G45*(1-$G$11)</f>
         <v/>
       </c>
       <c r="H50" s="42">
-        <f>H45*(1-'NOPAT Bridge'!F$39)</f>
+        <f>H45*(1-$G$11)</f>
         <v/>
       </c>
     </row>
@@ -2729,15 +2728,15 @@
         </is>
       </c>
       <c r="F51" s="42">
-        <f>F46*(1-'NOPAT Bridge'!G$39)</f>
+        <f>F46*(1-$G$11)</f>
         <v/>
       </c>
       <c r="G51" s="42">
-        <f>'NOPAT Bridge'!G41</f>
+        <f>G46*(1-$G$11)</f>
         <v/>
       </c>
       <c r="H51" s="42">
-        <f>H46*(1-'NOPAT Bridge'!G$39)</f>
+        <f>H46*(1-$G$11)</f>
         <v/>
       </c>
     </row>
@@ -2748,15 +2747,15 @@
         </is>
       </c>
       <c r="F52" s="42">
-        <f>F47*(1-'NOPAT Bridge'!H$39)</f>
+        <f>F47*(1-$G$11)</f>
         <v/>
       </c>
       <c r="G52" s="42">
-        <f>'NOPAT Bridge'!H41</f>
+        <f>G47*(1-$G$11)</f>
         <v/>
       </c>
       <c r="H52" s="42">
-        <f>H47*(1-'NOPAT Bridge'!H$39)</f>
+        <f>H47*(1-$G$11)</f>
         <v/>
       </c>
     </row>
@@ -2767,15 +2766,15 @@
         </is>
       </c>
       <c r="F53" s="42">
-        <f>F48*(1-'NOPAT Bridge'!I$39)</f>
+        <f>F48*(1-$G$11)</f>
         <v/>
       </c>
       <c r="G53" s="42">
-        <f>'NOPAT Bridge'!I41</f>
+        <f>G48*(1-$G$11)</f>
         <v/>
       </c>
       <c r="H53" s="42">
-        <f>H48*(1-'NOPAT Bridge'!I$39)</f>
+        <f>H48*(1-$G$11)</f>
         <v/>
       </c>
     </row>
@@ -2786,15 +2785,15 @@
         </is>
       </c>
       <c r="F54" s="42">
-        <f>F49*(1-'NOPAT Bridge'!J$39)</f>
+        <f>F49*(1-$G$11)</f>
         <v/>
       </c>
       <c r="G54" s="42">
-        <f>'NOPAT Bridge'!J41</f>
+        <f>G49*(1-$G$11)</f>
         <v/>
       </c>
       <c r="H54" s="42">
-        <f>H49*(1-'NOPAT Bridge'!J$39)</f>
+        <f>H49*(1-$G$11)</f>
         <v/>
       </c>
     </row>
@@ -7337,1193 +7336,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J45"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>NOPAT bridge</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
-      <c r="G1" s="13" t="n"/>
-      <c r="H1" s="13" t="n"/>
-      <c r="I1" s="13" t="n"/>
-      <c r="J1" s="13" t="n"/>
-    </row>
-    <row r="2">
-      <c r="B2" s="51" t="n"/>
-      <c r="C2" s="51" t="inlineStr">
-        <is>
-          <t>Source (click)</t>
-        </is>
-      </c>
-      <c r="D2" s="51" t="n"/>
-      <c r="E2" s="71" t="inlineStr">
-        <is>
-          <t>FY2025A</t>
-        </is>
-      </c>
-      <c r="F2" s="72" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="G2" s="72" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="H2" s="72" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="I2" s="72" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="J2" s="72" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="52" t="inlineStr">
-        <is>
-          <t>NOPAT bridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="26" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="52" t="inlineStr">
-        <is>
-          <t>Driver assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>SBC add-back (0)</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K): stock-based compensation</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="26" t="n"/>
-    </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Store-channel EBIT margin %</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: company-operated stores net revenue</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="20" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="I9" s="20" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="J9" s="20" t="n">
-        <v>0.186</v>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>E-commerce EBIT margin %</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: e-commerce net revenue</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="20" t="n">
-        <v>0.236</v>
-      </c>
-      <c r="F10" s="20" t="n">
-        <v>0.236</v>
-      </c>
-      <c r="G10" s="20" t="n">
-        <v>0.236</v>
-      </c>
-      <c r="H10" s="20" t="n">
-        <v>0.236</v>
-      </c>
-      <c r="I10" s="20" t="n">
-        <v>0.236</v>
-      </c>
-      <c r="J10" s="20" t="n">
-        <v>0.236</v>
-      </c>
-    </row>
-    <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Other-channels EBIT margin %</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: other channels (residual)</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="20" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="F11" s="20" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="G11" s="20" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="H11" s="20" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="I11" s="20" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="J11" s="20" t="n">
-        <v>0.091</v>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Terminal marginal tax rate</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="n"/>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F12" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G12" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I12" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J12" s="20" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>R&amp;D amortization period (years)</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge: capitalization convention</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="H13" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="I13" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="J13" s="40" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" hidden="1" outlineLevel="1">
-      <c r="A15" s="73" t="inlineStr">
-        <is>
-          <t>Reported EBIT adjustments</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Reported operating income (EBIT)</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: Income from operations</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="74" t="n">
-        <v>2210615</v>
-      </c>
-      <c r="F16" s="75">
-        <f>Scenarios!G45</f>
-        <v/>
-      </c>
-      <c r="G16" s="75">
-        <f>Scenarios!G46</f>
-        <v/>
-      </c>
-      <c r="H16" s="75">
-        <f>Scenarios!G47</f>
-        <v/>
-      </c>
-      <c r="I16" s="75">
-        <f>Scenarios!G48</f>
-        <v/>
-      </c>
-      <c r="J16" s="75">
-        <f>Scenarios!G49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>+ Impairment / intangible amortization (add-back)</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: amortization of intangible assets</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="74" t="n">
-        <v>6961</v>
-      </c>
-      <c r="F17" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>+ Restructuring costs (add-back)</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: restructuring charges</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>+ Legal / M&amp;A one-offs (add-back)</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: SG&amp;A one-offs</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" hidden="1" outlineLevel="1" ht="42" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>+ Stock-based compensation (add-back only if flag = 1)</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K): stock-based compensation</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="75">
-        <f>62203*$E$7</f>
-        <v/>
-      </c>
-      <c r="F20" s="75">
-        <f>Scenarios!G25/11102600*62203*$E$7</f>
-        <v/>
-      </c>
-      <c r="G20" s="75">
-        <f>Scenarios!G26/11102600*62203*$E$7</f>
-        <v/>
-      </c>
-      <c r="H20" s="75">
-        <f>Scenarios!G27/11102600*62203*$E$7</f>
-        <v/>
-      </c>
-      <c r="I20" s="75">
-        <f>Scenarios!G28/11102600*62203*$E$7</f>
-        <v/>
-      </c>
-      <c r="J20" s="75">
-        <f>Scenarios!G29/11102600*62203*$E$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A21" s="23" t="inlineStr">
-        <is>
-          <t>Adjusted EBIT (Phase 1)</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="24" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="n"/>
-      <c r="F21" s="25">
-        <f>F16+F17+F18+F19+F20</f>
-        <v/>
-      </c>
-      <c r="G21" s="25">
-        <f>G16+G17+G18+G19+G20</f>
-        <v/>
-      </c>
-      <c r="H21" s="25">
-        <f>H16+H17+H18+H19+H20</f>
-        <v/>
-      </c>
-      <c r="I21" s="25">
-        <f>I16+I17+I18+I19+I20</f>
-        <v/>
-      </c>
-      <c r="J21" s="25">
-        <f>J16+J17+J18+J19+J20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" hidden="1" outlineLevel="1">
-      <c r="A22" s="73" t="inlineStr">
-        <is>
-          <t>Lease &amp; R&amp;D adjustments</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" hidden="1" outlineLevel="1" ht="42" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>+ Implied lease interest expense (reclass from rent)</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: interest on lease liabilities (supplemental)</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="74" t="n">
-        <v>1028</v>
-      </c>
-      <c r="F23" s="75">
-        <f>1028*(Scenarios!G25/11102600)</f>
-        <v/>
-      </c>
-      <c r="G23" s="75">
-        <f>1028*(Scenarios!G26/11102600)</f>
-        <v/>
-      </c>
-      <c r="H23" s="75">
-        <f>1028*(Scenarios!G27/11102600)</f>
-        <v/>
-      </c>
-      <c r="I23" s="75">
-        <f>1028*(Scenarios!G28/11102600)</f>
-        <v/>
-      </c>
-      <c r="J23" s="75">
-        <f>1028*(Scenarios!G29/11102600)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>+ Capitalize R&amp;D / software (current-year expense)</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n"/>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: R&amp;D / software expense</t>
-        </is>
-      </c>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>− Amortization of prior capitalized intangibles</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="n"/>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: intangible amortization</t>
-        </is>
-      </c>
-      <c r="D25" s="19" t="n"/>
-      <c r="E25" s="74" t="n">
-        <v>6961</v>
-      </c>
-      <c r="F25" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A26" s="23" t="inlineStr">
-        <is>
-          <t>EBIT after lease &amp; capitalization (Phase 2)</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="n"/>
-      <c r="C26" s="24" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="n"/>
-      <c r="F26" s="25">
-        <f>F21+F23+F24-F25</f>
-        <v/>
-      </c>
-      <c r="G26" s="25">
-        <f>G21+G23+G24-G25</f>
-        <v/>
-      </c>
-      <c r="H26" s="25">
-        <f>H21+H23+H24-H25</f>
-        <v/>
-      </c>
-      <c r="I26" s="25">
-        <f>I21+I23+I24-I25</f>
-        <v/>
-      </c>
-      <c r="J26" s="25">
-        <f>J21+J23+J24-J25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" hidden="1" outlineLevel="1">
-      <c r="A27" s="73" t="inlineStr">
-        <is>
-          <t>Channel EBIT mix</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Store-channel revenue</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n"/>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: store-channel revenue</t>
-        </is>
-      </c>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="74" t="n">
-        <v>5049744</v>
-      </c>
-      <c r="F28" s="75">
-        <f>'Revenue Drivers'!C31</f>
-        <v/>
-      </c>
-      <c r="G28" s="75">
-        <f>'Revenue Drivers'!D31</f>
-        <v/>
-      </c>
-      <c r="H28" s="75">
-        <f>'Revenue Drivers'!E31</f>
-        <v/>
-      </c>
-      <c r="I28" s="75">
-        <f>'Revenue Drivers'!F31</f>
-        <v/>
-      </c>
-      <c r="J28" s="75">
-        <f>'Revenue Drivers'!G31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>E-commerce revenue</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n"/>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: e-commerce revenue</t>
-        </is>
-      </c>
-      <c r="D29" s="19" t="n"/>
-      <c r="E29" s="74" t="n">
-        <v>4918697</v>
-      </c>
-      <c r="F29" s="75">
-        <f>'Revenue Drivers'!C41</f>
-        <v/>
-      </c>
-      <c r="G29" s="75">
-        <f>'Revenue Drivers'!D41</f>
-        <v/>
-      </c>
-      <c r="H29" s="75">
-        <f>'Revenue Drivers'!E41</f>
-        <v/>
-      </c>
-      <c r="I29" s="75">
-        <f>'Revenue Drivers'!F41</f>
-        <v/>
-      </c>
-      <c r="J29" s="75">
-        <f>'Revenue Drivers'!G41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Other channels revenue</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="n"/>
-      <c r="C30" s="18" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: other channels revenue</t>
-        </is>
-      </c>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="74" t="n">
-        <v>1134159</v>
-      </c>
-      <c r="F30" s="75">
-        <f>'Revenue Drivers'!C45</f>
-        <v/>
-      </c>
-      <c r="G30" s="75">
-        <f>'Revenue Drivers'!D45</f>
-        <v/>
-      </c>
-      <c r="H30" s="75">
-        <f>'Revenue Drivers'!E45</f>
-        <v/>
-      </c>
-      <c r="I30" s="75">
-        <f>'Revenue Drivers'!F45</f>
-        <v/>
-      </c>
-      <c r="J30" s="75">
-        <f>'Revenue Drivers'!G45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Store-channel EBIT (= Rev × store margin)</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="n"/>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: company-operated stores net revenue</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="75" t="n">
-        <v>939252.384</v>
-      </c>
-      <c r="F31" s="75">
-        <f>F28*E$9</f>
-        <v/>
-      </c>
-      <c r="G31" s="75">
-        <f>G28*E$9</f>
-        <v/>
-      </c>
-      <c r="H31" s="75">
-        <f>H28*E$9</f>
-        <v/>
-      </c>
-      <c r="I31" s="75">
-        <f>I28*E$9</f>
-        <v/>
-      </c>
-      <c r="J31" s="75">
-        <f>J28*E$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>E-commerce EBIT (= Rev × e-comm margin)</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="n"/>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: e-commerce net revenue</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="75" t="n">
-        <v>1160812.492</v>
-      </c>
-      <c r="F32" s="75">
-        <f>F29*E$10</f>
-        <v/>
-      </c>
-      <c r="G32" s="75">
-        <f>G29*E$10</f>
-        <v/>
-      </c>
-      <c r="H32" s="75">
-        <f>H29*E$10</f>
-        <v/>
-      </c>
-      <c r="I32" s="75">
-        <f>I29*E$10</f>
-        <v/>
-      </c>
-      <c r="J32" s="75">
-        <f>J29*E$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1" ht="56" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>Other-channels EBIT (= Rev × other margin)</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: other channels (residual)</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="75" t="n">
-        <v>103208.469</v>
-      </c>
-      <c r="F33" s="75">
-        <f>F30*E$11</f>
-        <v/>
-      </c>
-      <c r="G33" s="75">
-        <f>G30*E$11</f>
-        <v/>
-      </c>
-      <c r="H33" s="75">
-        <f>H30*E$11</f>
-        <v/>
-      </c>
-      <c r="I33" s="75">
-        <f>I30*E$11</f>
-        <v/>
-      </c>
-      <c r="J33" s="75">
-        <f>J30*E$11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A34" s="23" t="inlineStr">
-        <is>
-          <t>Channel EBIT (sum of sector EBIT)</t>
-        </is>
-      </c>
-      <c r="B34" s="17" t="n"/>
-      <c r="C34" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: sector EBIT subtotal</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="n"/>
-      <c r="F34" s="70">
-        <f>F31+F32+F33+Scenarios!G7</f>
-        <v/>
-      </c>
-      <c r="G34" s="70">
-        <f>G31+G32+G33</f>
-        <v/>
-      </c>
-      <c r="H34" s="70">
-        <f>H31+H32+H33</f>
-        <v/>
-      </c>
-      <c r="I34" s="70">
-        <f>I31+I32+I33</f>
-        <v/>
-      </c>
-      <c r="J34" s="70">
-        <f>J31+J32+J33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A35" s="23" t="inlineStr">
-        <is>
-          <t>EBIT after channel mix (Phase 3)</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="24" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="76" t="n">
-        <v>2203273.345</v>
-      </c>
-      <c r="F35" s="25">
-        <f>F34</f>
-        <v/>
-      </c>
-      <c r="G35" s="25">
-        <f>G34</f>
-        <v/>
-      </c>
-      <c r="H35" s="25">
-        <f>H34</f>
-        <v/>
-      </c>
-      <c r="I35" s="25">
-        <f>I34</f>
-        <v/>
-      </c>
-      <c r="J35" s="25">
-        <f>J34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A36" s="23" t="inlineStr">
-        <is>
-          <t>Normalized EBIT (tax base for NOPAT)</t>
-        </is>
-      </c>
-      <c r="B36" s="17" t="n"/>
-      <c r="C36" s="24" t="inlineStr">
-        <is>
-          <t>Scenarios tab: base-case EBIT (forecast)</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="25">
-        <f>E21+E23+E24-E25</f>
-        <v/>
-      </c>
-      <c r="F36" s="25">
-        <f>Scenarios!G45</f>
-        <v/>
-      </c>
-      <c r="G36" s="25">
-        <f>Scenarios!G46</f>
-        <v/>
-      </c>
-      <c r="H36" s="25">
-        <f>Scenarios!G47</f>
-        <v/>
-      </c>
-      <c r="I36" s="25">
-        <f>Scenarios!G48</f>
-        <v/>
-      </c>
-      <c r="J36" s="25">
-        <f>Scenarios!G49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" hidden="1" outlineLevel="1">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Check vs Scenarios EBIT (base case)</t>
-        </is>
-      </c>
-      <c r="F37" s="75">
-        <f>F36-Scenarios!G45</f>
-        <v/>
-      </c>
-      <c r="G37" s="75">
-        <f>G36-Scenarios!G46</f>
-        <v/>
-      </c>
-      <c r="H37" s="75">
-        <f>H36-Scenarios!G47</f>
-        <v/>
-      </c>
-      <c r="I37" s="75">
-        <f>I36-Scenarios!G48</f>
-        <v/>
-      </c>
-      <c r="J37" s="75">
-        <f>J36-Scenarios!G49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" hidden="1" outlineLevel="1">
-      <c r="A38" s="73" t="inlineStr">
-        <is>
-          <t>Tax normalization</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>Operating effective tax rate (t_operating)</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="n"/>
-      <c r="C39" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: income tax &amp; interest expense</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="n"/>
-      <c r="E39" s="77" t="n">
-        <v>0.2946847649213503</v>
-      </c>
-      <c r="F39" s="32">
-        <f>0.29468476492135026+(F$12-0.29468476492135026)*1/5</f>
-        <v/>
-      </c>
-      <c r="G39" s="32">
-        <f>0.29468476492135026+(G$12-0.29468476492135026)*2/5</f>
-        <v/>
-      </c>
-      <c r="H39" s="32">
-        <f>0.29468476492135026+(H$12-0.29468476492135026)*3/5</f>
-        <v/>
-      </c>
-      <c r="I39" s="32">
-        <f>0.29468476492135026+(I$12-0.29468476492135026)*4/5</f>
-        <v/>
-      </c>
-      <c r="J39" s="32">
-        <f>0.29468476492135026+(J$12-0.29468476492135026)*5/5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Unlevered tax on normalized EBIT</t>
-        </is>
-      </c>
-      <c r="B40" s="17" t="n"/>
-      <c r="C40" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: unlevered tax expense</t>
-        </is>
-      </c>
-      <c r="D40" s="19" t="n"/>
-      <c r="F40" s="75">
-        <f>F36*F39</f>
-        <v/>
-      </c>
-      <c r="G40" s="75">
-        <f>G36*G39</f>
-        <v/>
-      </c>
-      <c r="H40" s="75">
-        <f>H36*H39</f>
-        <v/>
-      </c>
-      <c r="I40" s="75">
-        <f>I36*I39</f>
-        <v/>
-      </c>
-      <c r="J40" s="75">
-        <f>J36*J39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" collapsed="1" ht="28" customHeight="1">
-      <c r="A41" s="23" t="inlineStr">
-        <is>
-          <t>NORMALIZED NOPAT</t>
-        </is>
-      </c>
-      <c r="B41" s="17" t="n"/>
-      <c r="C41" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: normalized NOPAT</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="n"/>
-      <c r="F41" s="25">
-        <f>F36-F40</f>
-        <v/>
-      </c>
-      <c r="G41" s="25">
-        <f>G36-G40</f>
-        <v/>
-      </c>
-      <c r="H41" s="25">
-        <f>H36-H40</f>
-        <v/>
-      </c>
-      <c r="I41" s="25">
-        <f>I36-I40</f>
-        <v/>
-      </c>
-      <c r="J41" s="25">
-        <f>J36-J40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="61" t="inlineStr">
-        <is>
-          <t>6. Tariff refund (Scenarios)</t>
-        </is>
-      </c>
-      <c r="B43" s="79" t="n"/>
-      <c r="C43" s="79" t="inlineStr">
-        <is>
-          <t>EBIT = Rev × 13.2% only (no refund).</t>
-        </is>
-      </c>
-      <c r="D43" s="79" t="n"/>
-      <c r="F43" s="80" t="inlineStr">
-        <is>
-          <t>Scenarios EBIT (FY26)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="126" t="inlineStr">
-        <is>
-          <t>FY26 EBIT adjusted for one-time tariff refund. Base/Bear/Bull paths link to normalized NOPAT using a flat operating tax rate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="26" t="n"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId20"/>
-    <hyperlink ref="C28" location="'Revenue Drivers'!B31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId21"/>
-    <hyperlink ref="C29" location="'Revenue Drivers'!B41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId22"/>
-    <hyperlink ref="C30" location="'Revenue Drivers'!B45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId29"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <outlinePr applyStyles="1" summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -8615,11 +7427,7 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="38" t="n"/>
-      <c r="C4" s="85" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab</t>
-        </is>
-      </c>
+      <c r="C4" s="85" t="n"/>
       <c r="D4" s="85" t="inlineStr">
         <is>
           <t>Revenue Drivers tab</t>
@@ -8887,27 +7695,27 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Less: unlevered tax (t_operating from NOPAT Bridge)</t>
+          <t>Less: unlevered tax (cash tax rate)</t>
         </is>
       </c>
       <c r="F13" s="75">
-        <f>-'NOPAT Bridge'!F40</f>
+        <f>-F11*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="G13" s="75">
-        <f>-'NOPAT Bridge'!G40</f>
+        <f>-G11*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="H13" s="75">
-        <f>-'NOPAT Bridge'!H40</f>
+        <f>-H11*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="I13" s="75">
-        <f>-'NOPAT Bridge'!I40</f>
+        <f>-I11*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="J13" s="75">
-        <f>-'NOPAT Bridge'!J40</f>
+        <f>-J11*Scenarios!$G$11</f>
         <v/>
       </c>
     </row>
@@ -10188,23 +8996,23 @@
         <v>1579183</v>
       </c>
       <c r="F77" s="75">
-        <f>('NOPAT Bridge'!F36-'NOPAT Bridge'!F23)*(1-'NOPAT Bridge'!F$39)</f>
+        <f>F14</f>
         <v/>
       </c>
       <c r="G77" s="75">
-        <f>('NOPAT Bridge'!G36-'NOPAT Bridge'!G23)*(1-'NOPAT Bridge'!G$39)</f>
+        <f>G14</f>
         <v/>
       </c>
       <c r="H77" s="75">
-        <f>('NOPAT Bridge'!H36-'NOPAT Bridge'!H23)*(1-'NOPAT Bridge'!H$39)</f>
+        <f>H14</f>
         <v/>
       </c>
       <c r="I77" s="75">
-        <f>('NOPAT Bridge'!I36-'NOPAT Bridge'!I23)*(1-'NOPAT Bridge'!I$39)</f>
+        <f>I14</f>
         <v/>
       </c>
       <c r="J77" s="75">
-        <f>('NOPAT Bridge'!J36-'NOPAT Bridge'!J23)*(1-'NOPAT Bridge'!J$39)</f>
+        <f>J14</f>
         <v/>
       </c>
     </row>
@@ -10612,7 +9420,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
-    <hyperlink ref="C4" location="'NOPAT Bridge'!A1"/>
     <hyperlink ref="D4" location="'Revenue Drivers'!A1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
@@ -10669,7 +9476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Remove SOURCES heading from Cover page
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -1196,11 +1196,7 @@
       <c r="B15" s="5" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>SOURCES</t>
-        </is>
-      </c>
+      <c r="B17" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="11" t="n"/>

</xml_diff>

<commit_message>
Fix Scenarios #DIV/0! and restore Revenue Drivers sources
- Replace self-referencing Scenarios! anchors with local $B$ cells
- Add FY25 revenue anchor B198; scale balance sheet off $B$198 not DCF
- Restore RD source labels and hyperlinks from unaltered model; unhide col J
- Stop hiding Revenue Drivers source columns in outline groups

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="54">
+  <fonts count="56">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -350,6 +350,16 @@
       <i val="1"/>
       <sz val="8"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -409,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -757,6 +767,11 @@
     <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="55" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1735,7 +1750,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2216,6 +2231,7 @@
         <v>0.75</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4218,6 +4234,7 @@
         <v/>
       </c>
     </row>
+    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4275,6 +4292,7 @@
         <v/>
       </c>
     </row>
+    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4282,6 +4300,7 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -5321,6 +5340,20 @@
     </row>
     <row r="193">
       <c r="A193" s="26" t="n"/>
+    </row>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>FY25 net revenue ($000)</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>11102600</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5364,7 +5397,8 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="10" max="11"/>
+    <col width="28" customWidth="1" min="10" max="11"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
     <col collapsed="1" width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -5450,7 +5484,7 @@
         </is>
       </c>
       <c r="I5" s="56" t="n"/>
-      <c r="J5" s="56" t="inlineStr">
+      <c r="J5" s="127" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -5492,7 +5526,7 @@
         </is>
       </c>
       <c r="I6" s="17" t="n"/>
-      <c r="J6" s="24" t="inlineStr">
+      <c r="J6" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -5609,7 +5643,7 @@
         </is>
       </c>
       <c r="I9" s="17" t="n"/>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -5650,7 +5684,7 @@
         </is>
       </c>
       <c r="I10" s="17" t="n"/>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -5767,7 +5801,7 @@
         </is>
       </c>
       <c r="I13" s="17" t="n"/>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -5808,7 +5842,7 @@
         </is>
       </c>
       <c r="I14" s="17" t="n"/>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -5925,7 +5959,7 @@
         </is>
       </c>
       <c r="I17" s="17" t="n"/>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -5961,7 +5995,7 @@
         <v/>
       </c>
       <c r="I18" s="17" t="n"/>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-stores formula</t>
         </is>
@@ -6044,12 +6078,13 @@
         </is>
       </c>
       <c r="I20" s="17" t="n"/>
-      <c r="J20" s="24" t="inlineStr">
+      <c r="J20" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-sqft formula</t>
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6099,7 +6134,7 @@
         </is>
       </c>
       <c r="I23" s="56" t="n"/>
-      <c r="J23" s="56" t="inlineStr">
+      <c r="J23" s="129" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -6305,7 +6340,7 @@
         </is>
       </c>
       <c r="I28" s="17" t="n"/>
-      <c r="J28" s="24" t="inlineStr">
+      <c r="J28" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: prior store-rev formula</t>
         </is>
@@ -6341,7 +6376,7 @@
         <v/>
       </c>
       <c r="I29" s="17" t="n"/>
-      <c r="J29" s="24" t="inlineStr">
+      <c r="J29" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: comp-store formula</t>
         </is>
@@ -6377,7 +6412,7 @@
         <v/>
       </c>
       <c r="I30" s="17" t="n"/>
-      <c r="J30" s="24" t="inlineStr">
+      <c r="J30" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: net-new-store formula</t>
         </is>
@@ -6413,7 +6448,7 @@
         <v/>
       </c>
       <c r="I31" s="17" t="n"/>
-      <c r="J31" s="24" t="inlineStr">
+      <c r="J31" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: store-channel formula</t>
         </is>
@@ -6520,6 +6555,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -6569,7 +6605,7 @@
         </is>
       </c>
       <c r="I37" s="56" t="n"/>
-      <c r="J37" s="56" t="inlineStr">
+      <c r="J37" s="129" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -6719,12 +6755,13 @@
         <v/>
       </c>
       <c r="I41" s="17" t="n"/>
-      <c r="J41" s="24" t="inlineStr">
+      <c r="J41" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: e-comm formula</t>
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -6774,7 +6811,7 @@
         </is>
       </c>
       <c r="I44" s="56" t="n"/>
-      <c r="J44" s="56" t="inlineStr">
+      <c r="J44" s="129" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -7073,6 +7110,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -7122,7 +7160,7 @@
         </is>
       </c>
       <c r="I54" s="56" t="n"/>
-      <c r="J54" s="56" t="inlineStr">
+      <c r="J54" s="129" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -7159,7 +7197,7 @@
         <v/>
       </c>
       <c r="I55" s="17" t="n"/>
-      <c r="J55" s="24" t="inlineStr">
+      <c r="J55" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-rev formula</t>
         </is>
@@ -7237,7 +7275,7 @@
         <v/>
       </c>
       <c r="I57" s="17" t="n"/>
-      <c r="J57" s="24" t="inlineStr">
+      <c r="J57" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance formula</t>
         </is>
@@ -7274,7 +7312,7 @@
         <v/>
       </c>
       <c r="I58" s="17" t="n"/>
-      <c r="J58" s="24" t="inlineStr">
+      <c r="J58" s="128" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance % formula</t>
         </is>
@@ -7289,40 +7327,74 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId67"/>
+    <hyperlink ref="J56" location="'Scenarios'!G25"/>
     <hyperlink ref="K56" location="'Scenarios'!G25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7871,7 +7943,7 @@
         </is>
       </c>
     </row>
-    <row r="20" hidden="1" outlineLevel="1" ht="150" customHeight="1">
+    <row r="20" outlineLevel="1" ht="150" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>DSO (days) — flat vs FY25</t>
@@ -7908,7 +7980,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" hidden="1" outlineLevel="1" ht="98" customHeight="1">
+    <row r="21" outlineLevel="1" ht="98" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Accounts receivable, net</t>
@@ -7945,7 +8017,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" hidden="1" outlineLevel="1" ht="150" customHeight="1">
+    <row r="22" outlineLevel="1" ht="150" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>DIO (days) — FY25 anchor, −1 day/yr</t>
@@ -7982,7 +8054,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" hidden="1" outlineLevel="1" ht="112" customHeight="1">
+    <row r="23" outlineLevel="1" ht="112" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Inventories</t>
@@ -8019,7 +8091,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="24" outlineLevel="1" ht="84" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t>DPO (days) — flat vs FY25</t>
@@ -8056,7 +8128,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="25" outlineLevel="1" ht="84" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Accounts payable</t>
@@ -8093,7 +8165,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="26" outlineLevel="1" ht="84" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Prepaid expenses (% of revenue)</t>
@@ -8130,7 +8202,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="27" outlineLevel="1" ht="84" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Prepaid expenses (other current assets)</t>
@@ -8167,7 +8239,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="28" outlineLevel="1" ht="84" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Accrued liabilities (% of revenue)</t>
@@ -8204,7 +8276,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="29" outlineLevel="1" ht="84" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Accrued liabilities and other</t>
@@ -8241,7 +8313,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+    <row r="30" outlineLevel="1" ht="42" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Current operating assets (AR + inv + prepaids)</t>
@@ -8275,7 +8347,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+    <row r="31" outlineLevel="1" ht="42" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Current operating liabilities (AP + accruals)</t>
@@ -8309,7 +8381,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+    <row r="32" outlineLevel="1" ht="42" customHeight="1">
       <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Net working capital</t>

</xml_diff>

<commit_message>
Set buybacks to $750M and replace WC float literals with FY25 formulas
- Scenarios F21/G21: 750,000 ($750M/yr bear/base per pitch deck)
- DSO, DIO, DPO, prepaid/accrual %: formula-linked to DCF FY25A
- DCF FY25 WC driver rows use same day/% formulas
- DCF E78 accretive EPS: =E77/E75 instead of pasted 14.1783...
- Number formats: 0.0 days, 0.0% for percentages

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -21,13 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="56">
     <font>
@@ -419,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -772,6 +773,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="54" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1137,13 +1144,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1151,6 +1159,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1165,6 +1174,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1172,6 +1182,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1193,6 +1204,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -1210,9 +1222,11 @@
     <row r="15">
       <c r="B15" s="5" t="n"/>
     </row>
+    <row r="16"/>
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="5" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" s="11" t="n"/>
     </row>
@@ -1317,6 +1331,7 @@
         <v>0.3</v>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1424,6 +1439,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1633,6 +1649,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1668,6 +1685,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2074,14 +2092,17 @@
         </is>
       </c>
       <c r="D15" s="19" t="n"/>
-      <c r="F15" s="39" t="n">
-        <v>6.267883648875038</v>
-      </c>
-      <c r="G15" s="39" t="n">
-        <v>6.267883648875038</v>
-      </c>
-      <c r="H15" s="39" t="n">
-        <v>6.267883648875038</v>
+      <c r="F15" s="130">
+        <f>(DCF!$E$21/DCF!$E$5)*365</f>
+        <v/>
+      </c>
+      <c r="G15" s="130">
+        <f>(DCF!$E$21/DCF!$E$5)*365</f>
+        <v/>
+      </c>
+      <c r="H15" s="130">
+        <f>(DCF!$E$21/DCF!$E$5)*365</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="140" customHeight="1">
@@ -2097,14 +2118,17 @@
         </is>
       </c>
       <c r="D16" s="19" t="n"/>
-      <c r="F16" s="39" t="n">
-        <v>128.8324100108167</v>
-      </c>
-      <c r="G16" s="39" t="n">
-        <v>128.8324100108167</v>
-      </c>
-      <c r="H16" s="39" t="n">
-        <v>128.8324100108167</v>
+      <c r="F16" s="130">
+        <f>(DCF!$E$23/DCF!$E$8)*365</f>
+        <v/>
+      </c>
+      <c r="G16" s="130">
+        <f>(DCF!$E$23/DCF!$E$8)*365</f>
+        <v/>
+      </c>
+      <c r="H16" s="130">
+        <f>(DCF!$E$23/DCF!$E$8)*365</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="70" customHeight="1">
@@ -2143,14 +2167,17 @@
         </is>
       </c>
       <c r="D18" s="19" t="n"/>
-      <c r="F18" s="39" t="n">
-        <v>25.10521290169407</v>
-      </c>
-      <c r="G18" s="39" t="n">
-        <v>25.10521290169407</v>
-      </c>
-      <c r="H18" s="39" t="n">
-        <v>25.10521290169407</v>
+      <c r="F18" s="130">
+        <f>(DCF!$E$25/DCF!$E$8)*365</f>
+        <v/>
+      </c>
+      <c r="G18" s="130">
+        <f>(DCF!$E$25/DCF!$E$8)*365</f>
+        <v/>
+      </c>
+      <c r="H18" s="130">
+        <f>(DCF!$E$25/DCF!$E$8)*365</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="84" customHeight="1">
@@ -2166,14 +2193,17 @@
         </is>
       </c>
       <c r="D19" s="19" t="n"/>
-      <c r="F19" s="20" t="n">
-        <v>0.05080692810692991</v>
-      </c>
-      <c r="G19" s="20" t="n">
-        <v>0.05080692810692991</v>
-      </c>
-      <c r="H19" s="20" t="n">
-        <v>0.05080692810692991</v>
+      <c r="F19" s="20">
+        <f>DCF!$E$27/DCF!$E$5</f>
+        <v/>
+      </c>
+      <c r="G19" s="20">
+        <f>DCF!$E$27/DCF!$E$5</f>
+        <v/>
+      </c>
+      <c r="H19" s="20">
+        <f>DCF!$E$27/DCF!$E$5</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="84" customHeight="1">
@@ -2189,14 +2219,17 @@
         </is>
       </c>
       <c r="D20" s="19" t="n"/>
-      <c r="F20" s="20" t="n">
-        <v>0.05971412101669879</v>
-      </c>
-      <c r="G20" s="20" t="n">
-        <v>0.05971412101669879</v>
-      </c>
-      <c r="H20" s="20" t="n">
-        <v>0.05971412101669879</v>
+      <c r="F20" s="20">
+        <f>DCF!$E$29/DCF!$E$5</f>
+        <v/>
+      </c>
+      <c r="G20" s="20">
+        <f>DCF!$E$29/DCF!$E$5</f>
+        <v/>
+      </c>
+      <c r="H20" s="20">
+        <f>DCF!$E$29/DCF!$E$5</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2206,10 +2239,10 @@
         </is>
       </c>
       <c r="F21" s="37" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="G21" s="37" t="n">
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="H21" s="37" t="n">
         <v>0</v>
@@ -7579,8 +7612,9 @@
         </is>
       </c>
       <c r="D7" s="19" t="n"/>
-      <c r="E7" s="77" t="n">
-        <v>0.566005440167168</v>
+      <c r="E7" s="77">
+        <f>(E5-E8)/E5</f>
+        <v/>
       </c>
       <c r="F7" s="20">
         <f>Scenarios!$G$14</f>
@@ -7737,7 +7771,7 @@
         </is>
       </c>
       <c r="E12" s="77" t="n">
-        <v>0.1991078666258354</v>
+        <v>0.199</v>
       </c>
       <c r="F12" s="32">
         <f>F11/F5</f>
@@ -7956,8 +7990,9 @@
         </is>
       </c>
       <c r="D20" s="19" t="n"/>
-      <c r="E20" s="88" t="n">
-        <v>6.267883648875038</v>
+      <c r="E20" s="131">
+        <f>(E21/E5)*365</f>
+        <v/>
       </c>
       <c r="F20" s="28">
         <f>Scenarios!G65</f>
@@ -8030,8 +8065,9 @@
         </is>
       </c>
       <c r="D22" s="19" t="n"/>
-      <c r="E22" s="88" t="n">
-        <v>128.8324100108167</v>
+      <c r="E22" s="131">
+        <f>(E23/E8)*365</f>
+        <v/>
       </c>
       <c r="F22" s="28">
         <f>Scenarios!G75</f>
@@ -8104,8 +8140,9 @@
         </is>
       </c>
       <c r="D24" s="19" t="n"/>
-      <c r="E24" s="88" t="n">
-        <v>25.10521290169407</v>
+      <c r="E24" s="131">
+        <f>(E25/E8)*365</f>
+        <v/>
       </c>
       <c r="F24" s="28">
         <f>Scenarios!G85</f>
@@ -8178,8 +8215,9 @@
         </is>
       </c>
       <c r="D26" s="19" t="n"/>
-      <c r="E26" s="77" t="n">
-        <v>0.05080692810692991</v>
+      <c r="E26" s="77">
+        <f>E27/E5</f>
+        <v/>
       </c>
       <c r="F26" s="20">
         <f>Scenarios!$G$19</f>
@@ -8252,8 +8290,9 @@
         </is>
       </c>
       <c r="D28" s="19" t="n"/>
-      <c r="E28" s="77" t="n">
-        <v>0.05971412101669879</v>
+      <c r="E28" s="77">
+        <f>E29/E5</f>
+        <v/>
       </c>
       <c r="F28" s="20">
         <f>Scenarios!$G$20</f>
@@ -8558,6 +8597,7 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="n"/>
     </row>
@@ -8772,6 +8812,8 @@
         <v/>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -8790,14 +8832,16 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
           <t>Annual repurchase budget ($000) — base case</t>
         </is>
       </c>
-      <c r="E65" s="37" t="n">
-        <v>500000</v>
+      <c r="E65" s="37">
+        <f>Scenarios!$G$21</f>
+        <v/>
       </c>
       <c r="F65" s="37">
         <f>$E$65</f>
@@ -8850,6 +8894,7 @@
         <v/>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -8934,6 +8979,7 @@
         <v/>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -9054,6 +9100,7 @@
         <v/>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -9090,8 +9137,9 @@
           <t>Accretive EPS ($/share) = Net income ÷ ending shares</t>
         </is>
       </c>
-      <c r="E78" s="101" t="n">
-        <v>14.1783354282636</v>
+      <c r="E78" s="101">
+        <f>E77/E75</f>
+        <v/>
       </c>
       <c r="F78" s="101">
         <f>F77/F75</f>
@@ -9114,6 +9162,7 @@
         <v/>
       </c>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -9192,6 +9241,7 @@
         <v/>
       </c>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -9298,6 +9348,8 @@
       </c>
       <c r="D94" s="26" t="n"/>
     </row>
+    <row r="95"/>
+    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -9716,6 +9768,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -10033,6 +10086,7 @@
         <v>407521</v>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="n"/>
     </row>
@@ -10110,6 +10164,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -10160,6 +10215,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -10249,6 +10305,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -10395,6 +10452,7 @@
         <v/>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Formula-link DCF E12 reported EBIT margin (=E11/E5)
Last remaining FY25-derived hardcoded float; completes WC/EBIT
decimal cleanup across all tabs.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -7770,8 +7770,9 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E12" s="77" t="n">
-        <v>0.199</v>
+      <c r="E12" s="77">
+        <f>E11/E5</f>
+        <v/>
       </c>
       <c r="F12" s="32">
         <f>F11/F5</f>

</xml_diff>

<commit_message>
Fix Scenarios #DIV/0! from corrupted DCF cell refs
A naive DCF!$E$5 → $B$198 replace mangled DCF!$E$50/51/55 into
$B$1980/81/85 on implied share price (row 132) and cash bridge (row 163).
Restore correct DCF links; use regex to prevent recurrence.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -1144,14 +1144,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="B2:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1159,7 +1158,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1172,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1182,7 +1179,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1204,7 +1200,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -1222,11 +1217,9 @@
     <row r="15">
       <c r="B15" s="5" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="5" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="11" t="n"/>
     </row>
@@ -1331,7 +1324,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1439,7 +1431,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1649,7 +1640,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1685,7 +1675,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2093,15 +2082,15 @@
       </c>
       <c r="D15" s="19" t="n"/>
       <c r="F15" s="130">
-        <f>(DCF!$E$21/DCF!$E$5)*365</f>
+        <f>(DCF!$E$21/$B$198)*365</f>
         <v/>
       </c>
       <c r="G15" s="130">
-        <f>(DCF!$E$21/DCF!$E$5)*365</f>
+        <f>(DCF!$E$21/$B$198)*365</f>
         <v/>
       </c>
       <c r="H15" s="130">
-        <f>(DCF!$E$21/DCF!$E$5)*365</f>
+        <f>(DCF!$E$21/$B$198)*365</f>
         <v/>
       </c>
     </row>
@@ -2194,15 +2183,15 @@
       </c>
       <c r="D19" s="19" t="n"/>
       <c r="F19" s="20">
-        <f>DCF!$E$27/DCF!$E$5</f>
+        <f>DCF!$E$27/$B$198</f>
         <v/>
       </c>
       <c r="G19" s="20">
-        <f>DCF!$E$27/DCF!$E$5</f>
+        <f>DCF!$E$27/$B$198</f>
         <v/>
       </c>
       <c r="H19" s="20">
-        <f>DCF!$E$27/DCF!$E$5</f>
+        <f>DCF!$E$27/$B$198</f>
         <v/>
       </c>
     </row>
@@ -2220,15 +2209,15 @@
       </c>
       <c r="D20" s="19" t="n"/>
       <c r="F20" s="20">
-        <f>DCF!$E$29/DCF!$E$5</f>
+        <f>DCF!$E$29/$B$198</f>
         <v/>
       </c>
       <c r="G20" s="20">
-        <f>DCF!$E$29/DCF!$E$5</f>
+        <f>DCF!$E$29/$B$198</f>
         <v/>
       </c>
       <c r="H20" s="20">
-        <f>DCF!$E$29/DCF!$E$5</f>
+        <f>DCF!$E$29/$B$198</f>
         <v/>
       </c>
     </row>
@@ -4294,15 +4283,15 @@
         </is>
       </c>
       <c r="F132" s="46">
-        <f>(F131+1807202-1798441)/111380</f>
+        <f>(F131+DCF!$E$50+DCF!$E$51)/DCF!$E$55</f>
         <v/>
       </c>
       <c r="G132" s="47">
-        <f>(G131+1807202-1798441)/111380</f>
+        <f>(G131+DCF!$E$50+DCF!$E$51)/DCF!$E$55</f>
         <v/>
       </c>
       <c r="H132" s="46">
-        <f>(H131+1807202-1798441)/111380</f>
+        <f>(H131+DCF!$E$50+DCF!$E$51)/DCF!$E$55</f>
         <v/>
       </c>
     </row>
@@ -4808,15 +4797,15 @@
         </is>
       </c>
       <c r="F163" s="42">
-        <f>1807202+F153+F158</f>
+        <f>DCF!$E$50+F153+F158</f>
         <v/>
       </c>
       <c r="G163" s="42">
-        <f>1807202+G153+G158</f>
+        <f>DCF!$E$50+G153+G158</f>
         <v/>
       </c>
       <c r="H163" s="42">
-        <f>1807202+H153+H158</f>
+        <f>DCF!$E$50+H153+H158</f>
         <v/>
       </c>
     </row>
@@ -5432,7 +5421,7 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="11"/>
     <col width="13" customWidth="1" min="11" max="11"/>
-    <col collapsed="1" width="36" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8598,7 +8587,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="n"/>
     </row>
@@ -8813,8 +8801,6 @@
         <v/>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -8833,7 +8819,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -8895,7 +8880,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -8980,7 +8964,6 @@
         <v/>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -9101,7 +9084,6 @@
         <v/>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -9163,7 +9145,6 @@
         <v/>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -9242,7 +9223,6 @@
         <v/>
       </c>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -9349,8 +9329,6 @@
       </c>
       <c r="D94" s="26" t="n"/>
     </row>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -9769,7 +9747,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -10087,7 +10064,6 @@
         <v>407521</v>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="n"/>
     </row>
@@ -10165,7 +10141,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -10216,7 +10191,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -10306,7 +10280,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -10453,7 +10426,6 @@
         <v/>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Label RD unit conversions; sync pitch deck to model18 DCF ($133.52)
- Revenue Drivers B2/C2: explicit unit labels for ×1M sessions and ÷1K revenue
- eval_model18.py: Python DCF evaluator for model18_wsp_formulas.xlsx
- pitch_values.json + LULU_Investment_Pitch_Deck.pptx updated to base $133.52,
  EPS FY30 $14.58, FY27 $10.10 (+33.5% upside)
- Fix Scenarios implied price formulas (DCF E50/51/55, not $B$1980/85)

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_humanized (1).xlsx
+++ b/LULU/model18_humanized (1).xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="169" formatCode="0.0x"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="56">
+  <fonts count="58">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -361,6 +361,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -420,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -779,6 +787,8 @@
     <xf numFmtId="170" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2253,7 +2263,6 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4256,7 +4265,6 @@
         <v/>
       </c>
     </row>
-    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4314,7 +4322,6 @@
         <v/>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4322,7 +4329,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -5363,10 +5369,6 @@
     <row r="193">
       <c r="A193" s="26" t="n"/>
     </row>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
@@ -5447,8 +5449,34 @@
           <t>FY2025A = FY25 reported figures (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
         </is>
       </c>
+      <c r="B2" s="132" t="inlineStr">
+        <is>
+          <t>×1,000,000 (sessions in millions → count)</t>
+        </is>
+      </c>
+      <c r="C2" s="132" t="inlineStr">
+        <is>
+          <t>÷1,000 ($ → $000 on this tab)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Unit conversions (drivers)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H3" s="133" t="inlineStr">
+        <is>
+          <t>see B2/C2</t>
+        </is>
+      </c>
       <c r="I3" s="51" t="n"/>
       <c r="J3" s="51" t="inlineStr">
         <is>
@@ -6106,7 +6134,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6577,7 +6604,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -6783,7 +6809,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -7132,7 +7157,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>

</xml_diff>